<commit_message>
Finalizando arquivo ecofit md
</commit_message>
<xml_diff>
--- a/calculo de prazo.xlsx
+++ b/calculo de prazo.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\filipe.asilva7\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\filipe.asilva7\Desktop\TIPI04\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E14C2370-CC19-4C28-9632-B76F970262CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F801390D-728D-40CE-A4CE-BAD6636955DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{B92F7740-6A5C-41E8-91CE-652BC96B7A09}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
   <si>
     <t>Etapas</t>
   </si>
@@ -69,6 +69,12 @@
   </si>
   <si>
     <t>dividido por 6</t>
+  </si>
+  <si>
+    <t>brinde</t>
+  </si>
+  <si>
+    <t>lucro por pessoa</t>
   </si>
 </sst>
 </file>
@@ -78,7 +84,7 @@
   <numFmts count="1">
     <numFmt numFmtId="44" formatCode="_-&quot;R$&quot;\ * #,##0.00_-;\-&quot;R$&quot;\ * #,##0.00_-;_-&quot;R$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -95,6 +101,14 @@
     </font>
     <font>
       <sz val="48"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="72"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
@@ -128,7 +142,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="44" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1"/>
@@ -138,6 +152,7 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="44" fontId="2" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="44" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="44" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Moeda" xfId="1" builtinId="4"/>
@@ -473,16 +488,20 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0EB47BCC-490F-462F-A570-762920841B63}">
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:F13"/>
   <sheetFormatPr defaultRowHeight="63.75" x14ac:dyDescent="1"/>
   <cols>
     <col min="1" max="1" width="76.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="58.28515625" style="2" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="89.85546875" style="2" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="36" style="1" customWidth="1"/>
     <col min="4" max="4" width="58.28515625" style="2" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="9.140625" style="1"/>
     <col min="6" max="6" width="58.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="16384" width="9.140625" style="1"/>
+    <col min="7" max="8" width="9.140625" style="1"/>
+    <col min="9" max="9" width="33" style="1" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="9.140625" style="1"/>
+    <col min="11" max="11" width="28" style="1" bestFit="1" customWidth="1"/>
+    <col min="12" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="1">
@@ -497,15 +516,8 @@
       <c r="A2" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B2" s="2">
-        <v>0</v>
-      </c>
-      <c r="C2" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D2" s="5">
-        <f>B8*0.3</f>
-        <v>5250</v>
+      <c r="B2" s="2" t="s">
+        <v>11</v>
       </c>
       <c r="F2" s="2"/>
     </row>
@@ -514,7 +526,7 @@
         <v>4</v>
       </c>
       <c r="B3" s="2">
-        <v>0</v>
+        <v>17500</v>
       </c>
       <c r="F3" s="2"/>
     </row>
@@ -523,7 +535,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="2">
-        <v>0</v>
+        <v>14000</v>
       </c>
       <c r="F4" s="2"/>
     </row>
@@ -548,30 +560,30 @@
         <v>2</v>
       </c>
       <c r="B7" s="2">
-        <v>0</v>
+        <v>3000</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="1">
       <c r="A8" s="3"/>
       <c r="B8" s="2">
         <f>SUM(B2:B7)</f>
-        <v>17500</v>
+        <v>52000</v>
       </c>
       <c r="C8" s="6"/>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="1">
       <c r="B9" s="2">
-        <f>D2</f>
-        <v>5250</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="1">
-      <c r="A10" s="1" t="s">
+        <f>B12</f>
+        <v>15600</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" ht="93.75" x14ac:dyDescent="1.4">
+      <c r="A10" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="B10" s="2">
+      <c r="B10" s="7">
         <f>B8+B9</f>
-        <v>22750</v>
+        <v>67600</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="1">
@@ -580,7 +592,25 @@
       </c>
       <c r="B11" s="2">
         <f>B10/6</f>
-        <v>3791.6666666666665</v>
+        <v>11266.666666666666</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="1">
+      <c r="A12" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="B12" s="5">
+        <f>B8*0.3</f>
+        <v>15600</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="1">
+      <c r="A13" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B13" s="2">
+        <f>B12/6</f>
+        <v>2600</v>
       </c>
     </row>
   </sheetData>

</xml_diff>